<commit_message>
21-04_14-18 Reduce the codebase
</commit_message>
<xml_diff>
--- a/data/sample_dataset.xlsx
+++ b/data/sample_dataset.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="dataset" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,554 +430,182 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kết quả của việc chia 8 cho $\frac{1}{8}$ là bao nhiêu?</t>
+          <t>Tiệm bánh pizza bán pizza nhỏ với giá 2 đô la và pizza lớn với giá 8 đô la. Họ đã bán được 40 đô la tiền pizza. Nếu họ bán 8 chiếc pizza nhỏ thì họ đã bán được bao nhiêu chiếc pizza lớn?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Để chia cho một phân số, chúng ta nhân với nghịch đảo của nó. Vì vậy, chúng ta có $8 \div \frac{1}{8} = 8 \cdot \frac{8}{1} = \boxed{64}$. Đáp án là: 64</t>
+          <t>Nếu tiệm bánh pizza bán 8 chiếc pizza nhỏ với giá 2 đô la mỗi chiếc thì họ kiếm được 8 * 2 đô la = 16 đô la từ những chiếc pizza nhỏ. Họ đã bán được tổng cộng 40 đô la tiền pizza, vì vậy số tiền còn lại phải đến từ những chiếc pizza lớn. Số tiền làm được từ những chiếc pizza lớn là $40 - $16 = $24. Vì mỗi chiếc bánh pizza lớn có giá 8 đô la nên họ phải bán được 24 đô la / 8 đô la = 3 chiếc bánh pizza lớn. Vì vậy, họ đã bán được 3 chiếc pizza lớn. ####3 Đáp án là: 3</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cho rằng (3,17) và (9,-4) là hai đỉnh đối diện của một hình chữ nhật, tổng tọa độ y của hai đỉnh còn lại là bao nhiêu?</t>
+          <t>Sau khi nướng 200 chiếc bánh nhân thịt trong một ngày và bán với giá 20 USD mỗi chiếc, Du Chin dùng 3/5 số tiền bán được để mua nguyên liệu làm bánh nhân thịt cho ngày hôm sau. Đỗ Chín còn lại bao nhiêu tiền sau khi dành tiền mua nguyên liệu?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Các đỉnh đối diện của hình chữ nhật cách đều tâm hình chữ nhật. Tâm của hình chữ nhật là trung điểm của đoạn thẳng nối hai đỉnh đối diện. Trung điểm của đoạn thẳng nối (3,17) và (9,-4) là $\left(\frac{3+9}{2},\frac{17+(-4)}{2}\right ) = (6, \frac{13}{2})$. Hai đỉnh còn lại của hình chữ nhật cũng cách đều tâm hình chữ nhật. Do đó, tổng tọa độ y của hai đỉnh còn lại là $2 \times \frac{13}{2} = \boxed{13}$. Câu trả lời là: 13</t>
+          <t>Du Chin bán 200 cái bánh nhân thịt với giá 20$ mỗi cái, vậy tổng doanh thu là 200 x 20$ = $&lt;&lt;200*20=4000&gt;&gt;4000. Anh ấy sử dụng 3/5 doanh số bán hàng để mua nguyên liệu, vì vậy anh ấy chi 3/5 x $4000 = $&lt;&lt;3/5*4000=2400&gt;&gt;2400 cho nguyên liệu. Vì vậy, Du Chin còn lại $4000 - $2400 = $&lt;&lt;4000-2400=1600&gt;&gt;1600 sau khi dành tiền mua nguyên liệu. ####1600 Đáp án là: 1600</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nếu Diana kiếm được 150 đô la vào tháng 7, gấp 3 lần số tiền đó vào tháng 8 và gấp đôi số tiền cô ấy kiếm được vào tháng 8 vào tháng 9 thì tổng số tiền cô ấy kiếm được trong ba tháng này là bao nhiêu?</t>
+          <t>Trung bình của $x+6$, $6x+2$ và $2x+7$ là $4x-7$. $x$ là gì?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Diana kiếm được 150 USD trong tháng 7. Vào tháng 8, cô kiếm được gấp 3 lần số tiền đó nên cô kiếm được 3 * 150 USD = 450 USD. Vào tháng 9, cô kiếm được gấp đôi số tiền kiếm được trong tháng 8, do đó cô kiếm được 2 * 450 USD = 900 USD. Do đó, tổng số tiền cô ấy kiếm được trong ba tháng này là $150 + $450 + $900 = $1500. ####1500 Đáp án là: 1500</t>
+          <t>Trung bình cộng của ba số được tìm thấy bằng cách cộng chúng lại và chia cho 3. Vì vậy, chúng ta có phương trình: \[\frac{(x+6) + (6x+2) + (2x+7)}{3} = 4x-7.\] Rút gọn vế trái, ta có: \[\frac{9x+15}{3} = 4x-7.\] Nhân cả hai vế với 3 để loại bỏ phân số, ta có: \[ 9x+15 = 12x-21.\] Trừ 9x ở cả hai vế, ta có: \[15 = 3x-21.\] Cộng 21 vào cả hai vế, ta có: \[36 = 3x.\] Chia cả hai vế cho 3, ta có: \[x = 12.\] Vậy giá trị của x là $\boxed{12}$.Câu trả lời là: 12</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Giá trị của $81^{3/4}$ là bao nhiêu?</t>
+          <t>Trong tháng đầu năm, các gia đình đến thăm công viên quốc gia đã nhìn thấy động vật 26 lần. Trong tháng thứ hai, số lần nhìn thấy động vật nhiều gấp ba lần so với tháng Giêng. Trong tháng thứ ba, số lần nhìn thấy động vật giảm xuống còn một nửa so với tháng thứ hai. Tổng số lần các gia đình nhìn thấy một con vật trong ba tháng đầu năm là bao nhiêu?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chúng ta có thể viết lại $81$ thành $3^4$, vì vậy $81^{3/4} = (3^4)^{3/4} = 3^{4 \cdot \frac{3}{4}} = 3^ 3 = \boxed{27}$. Đáp án là: 27</t>
+          <t>Trong tháng đầu tiên, các gia đình đã nhìn thấy động vật 26 lần. Trong tháng thứ hai, số lần nhìn thấy động vật nhiều gấp ba lần so với tháng đầu tiên, do đó 26 x 3 = 78 lần nhìn thấy động vật. Trong tháng thứ ba, số lần nhìn thấy động vật giảm xuống còn một nửa so với tháng thứ hai, do đó 78/2 = 39 lần nhìn thấy động vật. Tổng số lần gia đình nhìn thấy một con vật trong 3 tháng đầu năm là 26 + 78 + 39 = 143. #### 143 Đáp án là: 143</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Nếu Bob lái xe trong 1,5 giờ với tốc độ 60 dặm/giờ và sau đó lái xe trong 2 giờ với tốc độ 45 dặm/giờ thì tổng quãng đường anh ấy đã đi trong 3,5 giờ đó là bao nhiêu?</t>
+          <t>Keenan cần viết một bài luận dài 1200 từ. Bài luận của cô ấy sẽ đến hạn vào lúc nửa đêm. Cô ấy viết 400 từ mỗi giờ trong hai giờ đầu tiên. Sau đó, cô viết 200 từ mỗi giờ. Cô ấy cần bắt đầu hoàn thành đúng thời hạn bao nhiêu giờ trước thời hạn?</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nếu Bob lái xe trong 1,5 giờ với tốc độ 60 mph thì quãng đường anh ấy đi được là 1,5 giờ * 60 mph = 90 dặm. Nếu sau đó Bob lái xe trong 2 giờ với tốc độ 45 dặm/giờ thì quãng đường anh ta đi được là 2 giờ * 45 dặm/giờ = 90 dặm. Do đó, tổng quãng đường Bob đi trong 3,5 giờ đó là 90 dặm + 90 dặm = 180 dặm. ####180 Đáp án là: 180</t>
+          <t>Keenan viết 400 từ mỗi giờ trong 2 giờ đầu, vậy cô ấy viết 400 x 2 = 800 từ trong 2 giờ đầu. Cô ấy cần viết tổng cộng 1200 từ, vậy cô ấy còn 1200 - 800 = 400 từ để viết. Sau 2 giờ đầu, cô ấy viết được 200 từ mỗi giờ, vậy cô ấy cần 400/200 = 2 giờ nữa để viết xong. Vì vậy, cô ấy cần bắt đầu viết trước thời hạn 2 + 2 = 4 tiếng để hoàn thành đúng hạn. ####4 Đáp án là: 4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bán kính của một hình cầu là đơn vị $p$ và bán kính của một bán cầu là đơn vị $2p$. Tỉ số giữa thể tích của hình cầu và thể tích của bán cầu là bao nhiêu?</t>
+          <t>Cho rằng (3,17) và (9,-4) là hai đỉnh đối diện của một hình chữ nhật, tổng tọa độ y của hai đỉnh còn lại là bao nhiêu?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Thể tích của hình cầu có bán kính $p$ là $\frac{4}{3}\pi p^3$ và thể tích của hình cầu có bán kính $2p$ là $\frac{2}{3}\pi (2p)^3$. Tỷ lệ giữa thể tích của hình cầu và thể tích của bán cầu là \[\frac{\frac{4}{3}\pi p^3}{\frac{2}{3}\pi (2p)^3 } = \frac{4}{3}\cdot \frac{1}{2^3}=\boxed{\frac{1}{4}}.\] Câu trả lời là: \frac{1}{4}</t>
+          <t>Các đỉnh đối diện của hình chữ nhật cách đều tâm hình chữ nhật. Tâm của hình chữ nhật là trung điểm của đoạn thẳng nối hai đỉnh đối diện. Trung điểm của đoạn thẳng nối (3,17) và (9,-4) là $\left(\frac{3+9}{2},\frac{17+(-4)}{2}\right ) = (6, \frac{13}{2})$. Hai đỉnh còn lại của hình chữ nhật cũng cách đều tâm hình chữ nhật. Do đó, tổng tọa độ y của hai đỉnh còn lại là $2 \times \frac{13}{2} = \boxed{13}$. Câu trả lời là: 13</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Jenna đang viền chiếc váy dạ hội của mình. Viền váy dài 3 feet. Mỗi mũi khâu mà Jenna thực hiện dài 1/4 inch. Nếu Jenna khâu 24 mũi mỗi phút thì Jenna mất bao nhiêu phút để viền váy?</t>
+          <t>Harry đang đi xe buýt về nhà. Anh ấy đã ngồi trên xe buýt được 15 phút và anh ấy biết chặng đường còn lại sẽ mất thêm 25 phút nữa. Quãng đường đi bộ từ bến xe buýt đến nhà anh ấy sẽ mất một nửa thời gian so với thời gian đi xe buýt. Tổng cộng Harry sẽ dành bao nhiêu phút để đi du lịch?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Đầu tiên, chúng ta cần chuyển đổi chiều dài của viền váy từ feet sang inch. Vì có 12 inch trong một foot nên chiều dài của viền áo tính bằng inch là 3 feet * 12 inch/foot = 36 inch. Tiếp theo, chúng ta cần tìm hiểu xem Jenna cần thực hiện bao nhiêu mũi khâu để viền chiếc váy. Vì mỗi mũi khâu dài 1/4 inch nên số mũi khâu cần thiết là 36 inch / (1/4 inch/mũi) = 36 inch * (4 mũi/1 inch) = 144 mũi. Cuối cùng, chúng ta cần xác định Jenna phải mất bao nhiêu phút để thực hiện 144 mũi khâu. Nếu Jenna thực hiện 24 mũi khâu mỗi phút thì cô ấy sẽ phải mất 144 mũi khâu / 24 mũi khâu/phút = 6 phút để viền váy. ####6 Đáp án là: 6</t>
+          <t>Harry đã ở trên xe buýt được 15 phút rồi. Phần còn lại của hành trình xe buýt sẽ mất thêm 25 phút nữa. Cho đến nay, Harry đã đi xe buýt tổng cộng 15 + 25 = 40 phút. Quãng đường đi bộ từ bến xe buýt đến nhà anh ấy sẽ mất một nửa thời gian so với thời gian đi xe buýt. Một nửa của 40 phút là 40/2 = 20 phút. Tổng cộng Harry sẽ mất 40 phút đi xe buýt + 20 phút đi bộ = 60 phút di chuyển. ####60 Đáp án là: 60</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Có bao nhiêu số thực $x$ là nghiệm của phương trình sau? \[ |x-1| = |x-2| + |x-3| \]</t>
+          <t>Jimmy muốn chơi trong bể bơi bơm hơi ở sân sau nhà mình. Bể bơi trống rỗng và gara bị khóa nên anh ta không thể dùng vòi để đổ nước vào bể. Anh ta tìm một cái xô 2 gallon và tính rằng phải mất 20 giây để đổ đầy nước từ vòi và mang nó đến bể nơi anh ta đổ nước vào. Nếu hồ chứa 84 gallon nước thì Jimmy sẽ mất bao nhiêu phút để đổ đầy hồ?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Chúng ta bắt đầu bằng việc xem xét các trường hợp khác nhau của giá trị $x$. Trường hợp 1: $x&lt;1$ Trong trường hợp này, cả $x-2$ và $x-3$ đều âm, vì vậy $|x-2| = -(x-2)$ và $|x-3| = -(x-3)$. Thay thế vào phương trình, chúng ta có $|x-1| = -(x-2) - (x-3)$. Đơn giản hóa, chúng ta nhận được $|x-1| = -2x + 5$. Vì $x&lt;1$, vế trái của phương trình là âm, trong khi vế phải là dương. Vì vậy, không có giải pháp nào trong trường hợp này. Trường hợp 2: $1 \leq x &lt; 2$ Trong trường hợp này, $x-2$ là âm, nhưng $x-3$ là dương. Thay thế vào phương trình, chúng ta có $|x-1| = -(x-2) + (x-3)$. Đơn giản hóa, chúng ta nhận được $|x-1| = -x - 1$. Phương trình này chỉ đúng khi $x = -2$. Vì $-2$ nằm trong khoảng $1 \leq x &lt; 2$, nên có một giải pháp trong trường hợp này. Trường hợp 3: $2 \leq x &lt; 3$ Trong trường hợp này, cả $x-2$ và $x-3$ đều dương, vì vậy $|x-2| = x-2$ và $|x-3| = x-3$. Thay thế vào phương trình, chúng ta có $|x-1| = (x-2) + (x-3)$. Đơn giản hóa, chúng ta nhận được $|x-1| = 2x - 5$. Chúng ta có thể viết lại phương trình này thành hai phương trình riêng biệt: $x-1 = 2x - 5$ và $x-1 = -(2x - 5)$. Giải các phương trình này, ta thấy $x = 4$ và $x = -2$. Tuy nhiên, $-2$ không nằm trong phạm vi $2 \leq x &lt; 3$, nên chỉ có một giải pháp trong trường hợp này. Trường hợp 4: $x \geq 3$ Trong trường hợp này, cả $x-2$ và $x-3$ đều dương, vì vậy $|x-2| = x-2$ và $|x-3| = x-3$. Thay thế vào phương trình, chúng ta có $|x-1| = (x-2) + (x-3)$. Đơn giản hóa, chúng ta nhận được $|x-1| = 2x - 5$. Vì $x \geq 3$, vế trái của phương trình là dương, trong khi vế phải là âm. Vì vậy, không có giải pháp nào trong trường hợp này. Tổng cộng có $\boxed{2}$ số thực $x$ là nghiệm của phương trình. Câu trả lời là: 2</t>
+          <t>Jimmy có thể đổ đầy bể bằng một thùng 2 gallon, vì vậy anh ta sẽ cần đổ đầy thùng 84/2 = 42 lần để đổ đầy bể. Jimmy mất 20 giây để đổ đầy thùng, do đó anh ấy sẽ mất 20 * 42 = 840 giây để đổ đầy bể. Vì một phút có 60 giây nên Jimmy sẽ mất 840/60 = 14 phút để làm đầy bể. ####14 Đáp án là: 14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sau khi ném một nửa trong số 18 viên sỏi ban đầu qua hồ, Marcus nhận thêm 30 viên sỏi từ Freddy. Bây giờ Marcus có tổng cộng bao nhiêu viên sỏi?</t>
+          <t>Jenna đang viền chiếc váy dạ hội của mình. Viền váy dài 3 feet. Mỗi mũi khâu mà Jenna thực hiện dài 1/4 inch. Nếu Jenna khâu 24 mũi mỗi phút thì Jenna mất bao nhiêu phút để viền váy?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ban đầu Marcus có 18 viên sỏi. Anh ta bỏ qua một nửa số viên sỏi, nên anh ta bỏ qua 18/2 = 9 viên sỏi. Sau khi bỏ qua, Marcus còn lại 18 - 9 = 9 viên sỏi. Sau đó, anh nhận thêm 30 viên sỏi từ Freddy. Cộng 30 viên sỏi vào 9 viên sỏi mà Marcus đã có, bây giờ anh ấy có tổng cộng 9 + 30 = 39 viên sỏi. #### 39 Đáp án là: 39</t>
+          <t>Đầu tiên, chúng ta cần chuyển đổi chiều dài của viền váy từ feet sang inch. Vì có 12 inch trong một foot nên chiều dài của viền áo tính bằng inch là 3 feet * 12 inch/foot = 36 inch. Tiếp theo, chúng ta cần tìm hiểu xem Jenna cần thực hiện bao nhiêu mũi khâu để viền chiếc váy. Vì mỗi mũi khâu dài 1/4 inch nên số mũi khâu cần thiết là 36 inch / (1/4 inch/mũi) = 36 inch * (4 mũi/1 inch) = 144 mũi. Cuối cùng, chúng ta cần xác định Jenna phải mất bao nhiêu phút để thực hiện 144 mũi khâu. Nếu Jenna thực hiện 24 mũi khâu mỗi phút thì cô ấy sẽ phải mất 144 mũi khâu / 24 mũi khâu/phút = 6 phút để viền váy. ####6 Đáp án là: 6</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Janele muốn tính trọng lượng trung bình của những con mèo của cô ấy. Cô ấy có 4 trong số đó. Hai cái đầu tiên nặng x pound mỗi cái. Quả thứ ba nặng 14,7 pound và quả thứ tư nặng 9,3 pound. Trọng số trung bình của chúng là 12. Giá trị của biến x chưa biết là bao nhiêu?</t>
+          <t>Nếu Brenda và chín người bạn của cô ấy dự định đặt một chiếc pizza, và mỗi người dự định ăn 2 lát, và mỗi chiếc pizza có 4 lát, thì họ nên đặt bao nhiêu chiếc pizza?</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Để giải bài toán này, chúng ta cần xác định giá trị của x, đại diện cho trọng lượng của hai con mèo đầu tiên. Hãy chia nhỏ thông tin đã cho: Số lượng mèo: 4 Trọng lượng của hai con mèo đầu tiên: x pound mỗi con Trọng lượng của con mèo thứ ba: 14,7 pound Trọng lượng của con mèo thứ tư: 9,3 pound Trọng lượng trung bình của những con mèo: 12 pound Chúng ta có thể thiết lập phương trình như sau: (Cân nặng của hai con mèo đầu tiên + Trọng lượng của con mèo thứ ba + Trọng lượng của con mèo thứ tư) / Số lượng mèo = Trọng lượng trung bình của những con mèo ((x + x) + 14,7 + 9,3) / 4 = 12 Hãy đơn giản hóa và giải x: (2x + 24) / 4 = 12 2x + 24 = 48 Để tách x, chúng ta trừ 24 từ cả hai vế của phương trình: 2x + 24 - 24 = 48 - 24 2x = 24 Để giải phương trình x, ta chia cả hai vế của phương trình cho 2: x = 24/2 x = 12 Giá trị của x là 12. #### 12 Đáp án là: 12</t>
+          <t>Brenda và 9 người bạn của cô ấy có tổng cộng 9 + 1 = 10 người. Mỗi người dự định ăn 2 lát nên sẽ cần tổng cộng 10 x 2 = 20 lát. Mỗi chiếc pizza có 4 lát nên họ sẽ cần đặt 20/4 = 5 chiếc pizza. ####5 Đáp án là: 5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nếu Luke đã làm được 33 ngôi sao giấy và cần đổ đầy 4 chai, mỗi chai cần 85 sao thì Luke cần làm thêm bao nhiêu ngôi sao nữa?</t>
+          <t>Diện tích của một hình tam giác là 600 feet vuông. Tìm độ cao tính bằng feet của tam giác nếu độ dài cạnh đáy tương ứng là 30 feet.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Luke cần đổ đầy 4 chai, mỗi chai cần 85 sao nên anh ấy cần tổng cộng 4 * 85 = 340 sao. Luke đã có 33 sao rồi nên anh ấy cần kiếm thêm 340 - 33 = 307 sao. Luke cần tạo thêm 307 ngôi sao nữa. #### 307 Đáp án là: 307</t>
+          <t>Diện tích của một tam giác được tính theo công thức $A = \frac{1}{2}bh$, trong đó $b$ là độ dài đáy và $h$ là đường cao. Chúng ta được biết rằng $A = 600$ feet vuông và $b = 30$ feet. Thay các giá trị này vào công thức, chúng ta có $600 = \frac{1}{2}(30)(h)$. Đơn giản hóa, chúng ta nhận được $600 = 15h$. Chia cả hai vế cho 15, ta thấy $h = \boxed{40}$ feet. Đáp án là: 40</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Số thập phân tương đương của số $\rm{A}03_{16}$ là bao nhiêu, trong đó 'các chữ số' từ A đến F biểu thị các giá trị 10, 11, 12, 13, 14 và 15 theo thứ tự?</t>
+          <t>Tìm nghịch đảo của ma trận \[\begin{pmatrix} 9 &amp; 18 \\ -6 &amp; -12 \end{pmatrix}.\]Nếu nghịch đảo không tồn tại thì nhập ma trận 0.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Số $\rm{A}03_{16}$ có thể được mở rộng thành $10 \cdot 16^2 + 0 \cdot 16^1 + 3 \cdot 16^0$. Đánh giá biểu thức này, chúng ta nhận được $10 \cdot 256 + 0 \cdot 16 + 3 \cdot 1 = 2560 + 3 = \boxed{2563}$. Đáp án là: 2563</t>
+          <t xml:space="preserve">
+Để tìm nghịch đảo của ma trận $2\times 2$ $\begin{pmatrix} a &amp; b \\ c &amp; d \end{pmatrix},$, chúng ta tính định thức $ad - bc.$ Nếu định thức khác 0 thì nghịch đảo được cho bởi \[\frac{1}{ad - bc} \begin{pmatrix} d &amp; -b \\ -c &amp; a \end{pmatrix}.\] Nếu định thức bằng 0 thì nghịch đảo sẽ không tồn tại. Trong trường hợp này, định thức là $9(-12) - 18(-6) = 0,$ nên nghịch đảo không tồn tại. Do đó, câu trả lời là ma trận 0 $\boxed{\begin{pmatrix} 0 &amp; 0 \\ 0 &amp; 0 \end{pmatrix}}.$Câu trả lời là: \begin{pmatrix}0&amp;0\0&amp;0\end{pmatrix}</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Diện tích của một hình tam giác là 600 feet vuông. Tìm độ cao tính bằng feet của tam giác nếu độ dài cạnh đáy tương ứng là 30 feet.</t>
+          <t>Jane chạy 3 km trong hai giờ. Tốc độ của cô ấy tính bằng mét trên phút là bao nhiêu?</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Diện tích của một tam giác được tính theo công thức $A = \frac{1}{2}bh$, trong đó $b$ là độ dài đáy và $h$ là đường cao. Chúng ta được biết rằng $A = 600$ feet vuông và $b = 30$ feet. Thay các giá trị này vào công thức, chúng ta có $600 = \frac{1}{2}(30)(h)$. Đơn giản hóa, chúng ta nhận được $600 = 15h$. Chia cả hai vế cho 15, ta thấy $h = \boxed{40}$ feet. Đáp án là: 40</t>
+          <t xml:space="preserve">
+Vì Jane chạy 3 km trong 2 giờ nên chúng ta cần đổi km sang mét và đổi giờ sang phút để tìm tốc độ của cô ấy bằng mét trên phút. Có 1000 mét trong 1 km, vậy 3 km bằng 3 * 1000 = 3000 mét. 1 giờ có 60 phút nên 2 giờ bằng 2 * 60 = 120 phút. Để tìm tốc độ của Jane tính bằng mét trên phút, chúng ta chia khoảng cách (tính bằng mét) cho thời gian (tính bằng phút). Vậy tốc độ của cô ấy là 3000 mét / 120 phút = 25 mét mỗi phút. #### 25 Đáp án là: 25</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Keenan cần viết một bài luận dài 1200 từ. Bài luận của cô ấy sẽ đến hạn vào lúc nửa đêm. Cô ấy viết 400 từ mỗi giờ trong hai giờ đầu tiên. Sau đó, cô viết 200 từ mỗi giờ. Cô ấy cần bắt đầu hoàn thành đúng thời hạn bao nhiêu giờ trước thời hạn?</t>
+          <t>Với bất kỳ số nguyên dương $n$ nào, giá trị của $n!$ là tích của các số nguyên dương $n$ đầu tiên. Ví dụ: 4 đô la! = 4\cdot 3\cdot 2\cdot 1 =24$. Ước chung lớn nhất của X và $7!$ là bao nhiêu? Nếu chúng ta biết câu trả lời cho câu hỏi trên là 120 thì giá trị của biến X chưa biết là bao nhiêu?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Keenan viết 400 từ mỗi giờ trong 2 giờ đầu, vậy cô ấy viết 400 x 2 = 800 từ trong 2 giờ đầu. Cô ấy cần viết tổng cộng 1200 từ, vậy cô ấy còn 1200 - 800 = 400 từ để viết. Sau 2 giờ đầu, cô ấy viết được 200 từ mỗi giờ, vậy cô ấy cần 400/200 = 2 giờ nữa để viết xong. Vì vậy, cô ấy cần bắt đầu viết trước thời hạn 2 + 2 = 4 tiếng để hoàn thành đúng hạn. ####4 Đáp án là: 4</t>
+          <t>Chúng ta muốn tìm giá trị của $X$ trong tình huống đã cho. Chúng ta được biết rằng ước số chung lớn nhất của $X$ và $7!$ là 120. Giai thừa của 7, ký hiệu là $7!$, là tích của 7 số nguyên dương đầu tiên: $7! = 7 \cdot 6 \cdot 5 \cdot 4 \cdot 3 \cdot 2 \cdot 1 = 5040$ Để tìm giá trị của $X$, chúng ta cần xác định các thừa số chung cho cả $X$ và $7!$ . Ước chung lớn nhất (GCD) là số nguyên dương lớn nhất chia cả hai số mà không để lại số dư. Hệ số nguyên tố của $7!$ là $2^4 \cdot 3^2 \cdot 5 \cdot 7$. Vì GCD của $X$ và $7!$ là 120, nên chúng ta có thể viết: $120 = 2^3 \cdot 3 \cdot 5$ Để tìm giá trị của $X$, chúng ta cần xác định các thừa số chung cho cả hai $120$ và $7!$. Chúng ta có thể chia $7!$ cho $120$ để tìm các thừa số còn lại: $\frac{7!}{120} = \frac{5040}{120} = 42$ Do đó, giá trị của $X$ là $42$. Lưu ý: GCD của hai số là tích của các thừa số nguyên tố chung được nâng lên số mũ thấp nhất. Trong trường hợp này, các thừa số nguyên tố chung giữa $X$ và $7!$ là $2^3$, $3$ và $5$. Câu trả lời là: 5</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Một hình chữ nhật không phải là hình vuông có kích thước nguyên. Số đơn vị vuông trong diện tích của nó bằng số lượng đơn vị trong chu vi của nó. Số đơn vị trong chu vi của hình chữ nhật này là bao nhiêu?</t>
+          <t>Grant đạt điểm cao hơn John 10 điểm trong bài kiểm tra toán. John nhận được số điểm gấp đôi Hunter, người đạt 45 điểm trong bài kiểm tra toán. Điểm kiểm tra của Grant là bao nhiêu?</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gọi kích thước của hình chữ nhật là $l$ và $w$. Diện tích của hình chữ nhật là $lw$ và chu vi là $2l + 2w$. Bài toán phát biểu rằng $lw = 2l + 2w$. Sắp xếp lại, ta có $lw - 2l - 2w = 0$. Sử dụng Thủ thuật phân tích nhân tử yêu thích của Simon, chúng ta có thể cộng 4 cho cả hai vế để được $(l - 2)(w - 2) = 4$. Các cặp thừa số nguyên dương của 4 là $(1, 4)$ và $(2, 2)$. Chúng ta có thể thiết lập hai trường hợp: Trường hợp 1: $l - 2 = 1$ và $w - 2 = 4$ Điều này cho chúng ta $l = 3$ và $w = 6$. Chu vi là $2l + 2w = 2(3) + 2(6) = 18$. Trường hợp 2: $l - 2 = 2$ và $w - 2 = 2$ Điều này cho ta $l = 4$ và $w = 4$. Chu vi là $2l + 2w = 2(4) + 2(4) = 16$. Chu vi có thể là 18 và 16, nhưng vì bài toán nói rằng hình chữ nhật không phải là hình vuông nên chu vi phải là $\boxed{18}$. Câu trả lời là: 18</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Jane chạy 3 km trong hai giờ. Tốc độ của cô ấy tính bằng mét trên phút là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
-Vì Jane chạy 3 km trong 2 giờ nên chúng ta cần đổi km sang mét và đổi giờ sang phút để tìm tốc độ của cô ấy bằng mét trên phút. Có 1000 mét trong 1 km, vậy 3 km bằng 3 * 1000 = 3000 mét. 1 giờ có 60 phút nên 2 giờ bằng 2 * 60 = 120 phút. Để tìm tốc độ của Jane tính bằng mét trên phút, chúng ta chia khoảng cách (tính bằng mét) cho thời gian (tính bằng phút). Vậy tốc độ của cô ấy là 3000 mét / 120 phút = 25 mét mỗi phút. #### 25 Đáp án là: 25</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Nếu $g(x) = x^2$ và $f(x) = 2x - 1$, giá trị của $f(g(2))$ là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Đầu tiên, chúng ta tìm $g(2)$ bằng cách thay $2$ vào hàm $g(x)$: $g(2) = 2^2 = 4$. Tiếp theo, chúng ta tìm $f(g(2))$ bằng cách thay $4$ vào hàm $f(x)$: $f(g(2)) = f(4) = 2(4) - 1 = 8 - 1 = \boxed{7}$. Câu trả lời là: 7</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Trong số 600 xe tại đại lý, 60% là xe hybrid và 40% trong số xe hybrid chỉ có một đèn pha. Có bao nhiêu chiếc xe hybrid trong đại lý còn nguyên cả hai đèn pha?</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Trong số 600 xe có 60% là xe hybrid nên có 600 * 0,60 = 360 xe hybrid. Trong số xe hybrid, 40% chỉ có một đèn pha, do đó có 360 * 0,40 = 144 xe hybrid chỉ có một đèn pha. Do đó, số xe hybrid còn nguyên cả hai đèn pha là 360 - 144 = 216. #### 216 Đáp án là: 216</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Trung bình của $x+6$, $6x+2$ và $2x+7$ là $4x-7$. $x$ là gì?</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Trung bình cộng của ba số được tìm thấy bằng cách cộng chúng lại và chia cho 3. Vì vậy, chúng ta có phương trình: \[\frac{(x+6) + (6x+2) + (2x+7)}{3} = 4x-7.\] Rút gọn vế trái, ta có: \[\frac{9x+15}{3} = 4x-7.\] Nhân cả hai vế với 3 để loại bỏ phân số, ta có: \[ 9x+15 = 12x-21.\] Trừ 9x ở cả hai vế, ta có: \[15 = 3x-21.\] Cộng 21 vào cả hai vế, ta có: \[36 = 3x.\] Chia cả hai vế cho 3, ta có: \[x = 12.\] Vậy giá trị của x là $\boxed{12}$.Câu trả lời là: 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Caleb mua 10 thùng kem và 4 thùng sữa chua đông lạnh. Mỗi hộp kem có giá 4 USD và mỗi hộp sữa chua đông lạnh có giá 1 USD. Caleb đã chi bao nhiêu cho kem so với sữa chua đông lạnh?</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Caleb mua 10 hộp kem và mỗi hộp có giá 4 đô la, vì vậy anh ấy đã chi 10 * 4 đô la = 40 đô la cho kem. Caleb cũng mua 4 hộp sữa chua đông lạnh và mỗi hộp có giá 1 đô la, vì vậy anh ấy đã chi 4 * 1 đô la = 4 đô la cho sữa chua đông lạnh. Sự chênh lệch về giá giữa kem và sữa chua đông lạnh là 40 USD - 4 USD = 36 USD. Vì vậy, Caleb đã chi 36 USD cho kem so với sữa chua đông lạnh. #### 36 Đáp án là: 36</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Jenny đạt được 95 điểm trong bài thi của mình. Điểm của Jason kém Jenny 25 điểm, còn điểm của Bob bằng một nửa điểm của Jason. Lớp của Bob là gì?</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Jenny đạt được điểm 95 trong bài thi của mình. Điểm của Jason kém Jenny 25 điểm nên điểm của Jason là 95 - 25 = 70. Điểm của Bob bằng một nửa điểm của Jason nên điểm của Bob là 70/2 = 35. Do đó, điểm của Bob là 35. #### 35 Đáp án là: 35</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Nếu Harper cần mua những món quà tri ân giáo viên dành cho các giáo viên của con cô ấy, trong đó con trai cô ấy có 3 giáo viên và con gái cô ấy có 4 giáo viên, và cô ấy đã chi tổng cộng 70 đô la cho những món quà, giá mỗi món quà là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Harper phải mua quà cho tổng cộng 3 + 4 = 7 giáo viên. Cô ấy đã chi tổng cộng 70 USD cho quà tặng, vì vậy giá của mỗi món quà là 70 USD / 7 = 10 USD. ####10 Đáp án là: 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Sau khi nướng 200 chiếc bánh nhân thịt trong một ngày và bán với giá 20 USD mỗi chiếc, Du Chin dùng 3/5 số tiền bán được để mua nguyên liệu làm bánh nhân thịt cho ngày hôm sau. Đỗ Chín còn lại bao nhiêu tiền sau khi dành tiền mua nguyên liệu?</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Du Chin bán 200 cái bánh nhân thịt với giá 20$ mỗi cái, vậy tổng doanh thu là 200 x 20$ = $&lt;&lt;200*20=4000&gt;&gt;4000. Anh ấy sử dụng 3/5 doanh số bán hàng để mua nguyên liệu, vì vậy anh ấy chi 3/5 x $4000 = $&lt;&lt;3/5*4000=2400&gt;&gt;2400 cho nguyên liệu. Vì vậy, Du Chin còn lại $4000 - $2400 = $&lt;&lt;4000-2400=1600&gt;&gt;1600 sau khi dành tiền mua nguyên liệu. ####1600 Đáp án là: 1600</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Tiệm bánh pizza bán pizza nhỏ với giá 2 đô la và pizza lớn với giá 8 đô la. Họ đã bán được 40 đô la tiền pizza. Nếu họ bán 8 chiếc pizza nhỏ thì họ đã bán được bao nhiêu chiếc pizza lớn?</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Nếu tiệm bánh pizza bán 8 chiếc pizza nhỏ với giá 2 đô la mỗi chiếc thì họ kiếm được 8 * 2 đô la = 16 đô la từ những chiếc pizza nhỏ. Họ đã bán được tổng cộng 40 đô la tiền pizza, vì vậy số tiền còn lại phải đến từ những chiếc pizza lớn. Số tiền làm được từ những chiếc pizza lớn là $40 - $16 = $24. Vì mỗi chiếc bánh pizza lớn có giá 8 đô la nên họ phải bán được 24 đô la / 8 đô la = 3 chiếc bánh pizza lớn. Vì vậy, họ đã bán được 3 chiếc pizza lớn. ####3 Đáp án là: 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Alicia phải mua vài cuốn sách cho năm học mới. Cô ấy mua x cuốn sách toán, 3 cuốn sách nghệ thuật và 6 cuốn sách khoa học, tổng cộng là 30$. Nếu cả hai cuốn sách toán và khoa học đều có giá 3 đô la mỗi cuốn thì giá của mỗi cuốn sách nghệ thuật là 2. Giá trị của biến x chưa biết là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Để giải bài toán này, chúng ta cần xác định giá trị của x, đại diện cho số sách toán mà Alicia mua. Hãy chia nhỏ thông tin đã cho: Số sách toán: x Số sách nghệ thuật: 3 Số sách khoa học: 6 Tổng chi phí: $30 Giá mỗi cuốn sách toán: $3 Giá mỗi cuốn sách khoa học: $3 Giá mỗi cuốn sách nghệ thuật: $2 Chúng ta có thể thiết lập phương trình như sau: Số sách toán * Giá một cuốn sách toán + Số sách nghệ thuật * Giá một cuốn sách nghệ thuật + Số sách khoa học * Giá mỗi cuốn sách khoa học = Tổng chi phí x * $3 + 3 * $2 + 6 * $3 = $30 Hãy đơn giản hóa và giải tìm x: $3x + $6 + $18 = $30 $3x + $24 = $30 Để tách x, chúng ta trừ $24 từ cả hai vế của phương trình: $3x + $24 - $24 = $30 - $24 $3 x = $6 Để giải x, chúng ta chia cả hai vế của phương trình cho $3: x = $6 / $3 x = 2 Giá trị của x là 2. #### 2 Đáp án là: 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Kết quả của $(5@3)-(3@5)$ là gì, trong đó $x@y = xy - 2x$?</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Chúng ta thay thế $x=5$ và $y=3$ vào biểu thức $x@y=xy-2x$ để tìm ra rằng $5@3=(5)(3)-2(5)=15-10=5$ . Tương tự, chúng ta thay thế $x=3$ và $y=5$ vào biểu thức $x@y=xy-2x$ để tìm ra rằng $3@5=(3)(5)-2(3)=15-6= 9 đô la. Do đó, $(5@3)-(3@5)=5-9=\boxed{-4}$. Câu trả lời là: -4</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Nếu giá của một chiếc iPhone ban đầu là 1000 USD và giảm 10% trong tháng đầu tiên và giảm thêm 20% trong tháng thứ hai thì giá iPhone sau tháng thứ hai là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Trong tháng đầu tiên, giá iPhone giảm 10% nên bây giờ là 1000 - (10/100 * 1000) = 1000 - 100 = 900 USD. Trong tháng thứ hai, giá giảm thêm 20% nên giá mới là 900 - (20/100 * 900) = 900 - 180 = 720 USD. Do đó, giá iPhone sau tháng thứ hai là 720 USD. ####720 Đáp án là: 720</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Nếu Roberto có bốn chiếc quần dài, bảy chiếc áo sơ mi và ba chiếc áo khoác, thì anh ấy có thể tạo ra bao nhiêu bộ trang phục độc đáo bằng cách kết hợp một chiếc quần dài, một chiếc áo sơ mi và một chiếc áo khoác?</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Với mỗi chiếc quần, Roberto có bảy chiếc áo sơ mi để lựa chọn. Với mỗi cách kết hợp quần và áo sơ mi, anh có ba lựa chọn áo khoác. Do đó, tổng số trang phục độc đáo là $4 \times 7 \times 3 = \boxed{84}$.Câu trả lời là: 84</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Với bất kỳ số nguyên dương $n$ nào, giá trị của $n!$ là tích của các số nguyên dương $n$ đầu tiên. Ví dụ: 4 đô la! = 4\cdot 3\cdot 2\cdot 1 =24$. Ước chung lớn nhất của X và $7!$ là bao nhiêu? Nếu chúng ta biết câu trả lời cho câu hỏi trên là 120 thì giá trị của biến X chưa biết là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Chúng ta muốn tìm giá trị của $X$ trong tình huống đã cho. Chúng ta được biết rằng ước số chung lớn nhất của $X$ và $7!$ là 120. Giai thừa của 7, ký hiệu là $7!$, là tích của 7 số nguyên dương đầu tiên: $7! = 7 \cdot 6 \cdot 5 \cdot 4 \cdot 3 \cdot 2 \cdot 1 = 5040$ Để tìm giá trị của $X$, chúng ta cần xác định các thừa số chung cho cả $X$ và $7!$ . Ước chung lớn nhất (GCD) là số nguyên dương lớn nhất chia cả hai số mà không để lại số dư. Hệ số nguyên tố của $7!$ là $2^4 \cdot 3^2 \cdot 5 \cdot 7$. Vì GCD của $X$ và $7!$ là 120, nên chúng ta có thể viết: $120 = 2^3 \cdot 3 \cdot 5$ Để tìm giá trị của $X$, chúng ta cần xác định các thừa số chung cho cả hai $120$ và $7!$. Chúng ta có thể chia $7!$ cho $120$ để tìm các thừa số còn lại: $\frac{7!}{120} = \frac{5040}{120} = 42$ Do đó, giá trị của $X$ là $42$. Lưu ý: GCD của hai số là tích của các thừa số nguyên tố chung được nâng lên số mũ thấp nhất. Trong trường hợp này, các thừa số nguyên tố chung giữa $X$ và $7!$ là $2^3$, $3$ và $5$. Câu trả lời là: 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Nếu một đa giác đều có chu vi 108 cm và mỗi cạnh là 12 cm thì đa giác đó có bao nhiêu cạnh?</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Nếu mỗi cạnh của đa giác có kích thước 12 cm thì chu vi của đa giác là $12n$ cm, trong đó $n$ là số cạnh. Chúng ta được biết chu vi là 108 cm, vì vậy chúng ta có phương trình $12n = 108$. Chia cả hai vế cho 12, ta thấy $n = 9$. Do đó, đa giác có các cạnh $\boxed{9}$. Câu trả lời là: 9</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Nếu ban đầu có 14 con sâu bướm trên cây và 4 quả trứng nữa nở ra trong khi 8 con sâu bướm mập mạp còn lại để làm kén thì trên cây còn lại bao nhiêu con sâu bướm?</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Nếu ban đầu trên cây có 14 con sâu, sau đó nở thêm 4 quả trứng nữa thì trên cây có tổng cộng 14 + 4 = 18 con sâu. Nếu để 8 con sâu mập béo tự làm kén thì số con sâu còn lại trên cây là 18 - 8 = 10. #### 10 Đáp án là: 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Đặt $a \bowtie b = a+\sqrt{b+\sqrt{b+\sqrt{b+...}}}$. Nếu $4\bowtie y = 10$, hãy tìm giá trị của $y$.</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Chúng ta có $4 \bowtie y = 4 + \sqrt{y+\sqrt{y+\sqrt{y+...}}} = 10$. Trừ 4 từ cả hai vế, chúng ta có $\sqrt{y+\sqrt{y+\sqrt{y+...}}} = 6$. Bình phương cả hai vế, ta có $y+\sqrt{y+\sqrt{y+...}} = 36$. Thay $\sqrt{y+\sqrt{y+\sqrt{y+...}}}$ bằng 6, chúng ta có $y+6=36$. Trừ 6 ở cả hai vế, chúng ta có $y=30$. Do đó, giá trị của $y$ là $\boxed{30}$. Câu trả lời là: 30</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Tìm nghịch đảo của ma trận \[\begin{pmatrix} 9 &amp; 18 \\ -6 &amp; -12 \end{pmatrix}.\]Nếu nghịch đảo không tồn tại thì nhập ma trận 0.</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
-Để tìm nghịch đảo của ma trận $2\times 2$ $\begin{pmatrix} a &amp; b \\ c &amp; d \end{pmatrix},$, chúng ta tính định thức $ad - bc.$ Nếu định thức khác 0 thì nghịch đảo được cho bởi \[\frac{1}{ad - bc} \begin{pmatrix} d &amp; -b \\ -c &amp; a \end{pmatrix}.\] Nếu định thức bằng 0 thì nghịch đảo sẽ không tồn tại. Trong trường hợp này, định thức là $9(-12) - 18(-6) = 0,$ nên nghịch đảo không tồn tại. Do đó, câu trả lời là ma trận 0 $\boxed{\begin{pmatrix} 0 &amp; 0 \\ 0 &amp; 0 \end{pmatrix}}.$Câu trả lời là: \begin{pmatrix}0&amp;0\0&amp;0\end{pmatrix}</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Năm 2004, có 60 đứa trẻ tham gia một buổi nấu ăn. Năm 2005, số trẻ em đến tham gia nấu ăn chỉ bằng một nửa so với năm 2004. Năm 2006, số trẻ em đến tham gia nấu ăn bằng 2/3 so với năm 2005. Có bao nhiêu trẻ em đến tham gia nấu ăn vào năm 2006?</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Năm 2005, số trẻ đến tham gia nấu ăn bằng một nửa so với năm 2004 nên có 60/2 = 30 trẻ vào năm 2005. Năm 2006, số trẻ đến tham gia nấu ăn bằng 2/3 so với năm 2005 nên có 30 trẻ. * 2/3 = 20 em năm 2006. Vậy có 20 em đến tham gia nấu ăn năm 2006. #### 20 Đáp án là: 20</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Evie đang thu thập vỏ sò ở bãi biển. Mỗi ngày cô thu thập được 10 chiếc vỏ sò yêu thích của mình. Hết 6 ngày, cô đưa cho anh trai 2 vỏ sò. Cô ấy còn lại bao nhiêu vỏ sò?</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Evie thu thập 10 vỏ sò mỗi ngày trong 6 ngày, vậy cô ấy có 10 * 6 = 60 vỏ sò. Cô đưa cho anh trai 2 vỏ sò, vậy cô còn lại 60 - 2 = 58 vỏ sò. ####58 Đáp án là: 58</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Harry đang đi xe buýt về nhà. Anh ấy đã ngồi trên xe buýt được 15 phút và anh ấy biết chặng đường còn lại sẽ mất thêm 25 phút nữa. Quãng đường đi bộ từ bến xe buýt đến nhà anh ấy sẽ mất một nửa thời gian so với thời gian đi xe buýt. Tổng cộng Harry sẽ dành bao nhiêu phút để đi du lịch?</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Harry đã ở trên xe buýt được 15 phút rồi. Phần còn lại của hành trình xe buýt sẽ mất thêm 25 phút nữa. Cho đến nay, Harry đã đi xe buýt tổng cộng 15 + 25 = 40 phút. Quãng đường đi bộ từ bến xe buýt đến nhà anh ấy sẽ mất một nửa thời gian so với thời gian đi xe buýt. Một nửa của 40 phút là 40/2 = 20 phút. Tổng cộng Harry sẽ mất 40 phút đi xe buýt + 20 phút đi bộ = 60 phút di chuyển. ####60 Đáp án là: 60</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Brianna bắt đầu với một túi 24 viên bi. Cô ấy làm mất x viên bi qua một cái lỗ trên túi. Sau đó, cô ấy đã cho đi số viên bi gấp đôi số bi đã làm mất qua lỗ trên túi. Cuối cùng, con chó của cô đã ăn được một nửa số viên bi mà Brianna đã làm mất qua lỗ trên túi. Brianna còn lại 10 viên bi.</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Để giải bài toán này, chúng ta cần xác định giá trị của x, biểu thị số viên bi mà Brianna bị mất qua lỗ trên túi. Hãy chia nhỏ thông tin đã cho: Số viên bi Brianna bắt đầu bằng: 24 Số viên bi Brianna bị mất qua lỗ trên túi: x Số viên bi Brianna đã cho đi: 2x Số viên bi mà con chó của Brianna đã ăn: (1/2)x Số Số viên bi Brianna còn lại: 10 Chúng ta có thể thiết lập phương trình như sau: Số viên bi Brianna bắt đầu - Số viên bi bị mất - Số viên bi đã cho đi - Số viên bi bị con chó ăn = Số viên bi còn lại 24 - x - 2x - (1/2)x = 10 Hãy đơn giản hóa và giải x: 24 - 3,5x = 10 Để tách x, chúng ta trừ 24 từ cả hai vế của phương trình: 24 - 24 - 3,5x = 10 - 24 -3,5x = -14 Để giải x ta chia cả hai vế của phương trình cho -3,5: x = -14 / -3,5 x = 4 Giá trị của x là 4. #### 4 Đáp án là: 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Số cơ sở ba $12012_3$ bằng cơ số mười nào?</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Ba số cơ số $12012_3$ có thể được mở rộng thành $1\cdot3^4 + 2\cdot3^3 + 0\cdot3^2 + 1\cdot3^1 + 2\cdot3^0$. Đánh giá biểu thức này, chúng ta thấy rằng $12012_3 = 81 + 54 + 0 + 3 + 2 = \boxed{140}$ trong cơ số mười. Đáp án là: 140</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Một ổ khóa vali có 3 mặt số, mỗi mặt có các chữ số $0, 1, 2,..., 9$. Có thể có bao nhiêu cách thiết lập khác nhau nếu cả ba chữ số phải khác nhau?</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Đối với mặt số đầu tiên, có 10 chữ số có thể lựa chọn. Đối với mặt số thứ hai, có 9 chữ số có thể còn lại để chọn (vì chúng ta không thể lặp lại chữ số từ mặt số thứ nhất). Đối với mặt số thứ ba, còn lại 8 chữ số để bạn lựa chọn. Do đó, tổng số cài đặt khác nhau là $10 \times 9 \times 8 = \boxed{720}$.Câu trả lời là: 720</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Nếu Nicky dành 20 phút chờ để lấy số ở DMV và tăng gấp bốn lần khoảng thời gian đó cộng thêm 14 phút chờ số của anh ấy được gọi, thì tổng thời gian anh ấy đã chờ đợi là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Nicky phải đợi 20 phút để lấy số. Anh ấy cũng dành gấp bốn lần thời gian đó để chờ gọi số của mình, tức là 20 x 4 = 80 phút. Ngoài ra, anh còn phải mất thêm 14 phút để chờ gọi đến số của mình. Do đó, tổng thời gian Nicky chờ đợi là 20 + 80 + 14 = 114 phút. ####114 Đáp án là: 114</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Ba người bạn của tôi và tôi ăn tối cùng nhau vào mỗi cuối tuần. Mỗi cuối tuần, hai người chúng tôi nấu ăn và hai người còn lại dọn dẹp sau đó. Có bao nhiêu cách khác nhau để chúng ta lựa chọn ai nấu ăn và ai dọn dẹp?</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Đầu tiên chúng ta cần chọn ra hai người sẽ nấu ăn. Điều này có thể được thực hiện theo các cách $\binom{4}{2}=6$. Sau khi chúng ta đã chọn xong người nấu ăn, hai người còn lại sẽ tự động được phân công dọn dẹp. Do đó, $\boxed{6}$ có nhiều cách khác nhau để chọn ai nấu và ai dọn dẹp. Câu trả lời là: 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Trong tháng đầu năm, các gia đình đến thăm công viên quốc gia đã nhìn thấy động vật 26 lần. Trong tháng thứ hai, số lần nhìn thấy động vật nhiều gấp ba lần so với tháng Giêng. Trong tháng thứ ba, số lần nhìn thấy động vật giảm xuống còn một nửa so với tháng thứ hai. Tổng số lần các gia đình nhìn thấy một con vật trong ba tháng đầu năm là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Trong tháng đầu tiên, các gia đình đã nhìn thấy động vật 26 lần. Trong tháng thứ hai, số lần nhìn thấy động vật nhiều gấp ba lần so với tháng đầu tiên, do đó 26 x 3 = 78 lần nhìn thấy động vật. Trong tháng thứ ba, số lần nhìn thấy động vật giảm xuống còn một nửa so với tháng thứ hai, do đó 78/2 = 39 lần nhìn thấy động vật. Tổng số lần gia đình nhìn thấy một con vật trong 3 tháng đầu năm là 26 + 78 + 39 = 143. #### 143 Đáp án là: 143</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Grant đạt điểm cao hơn John 10 điểm trong bài kiểm tra toán. John nhận được số điểm gấp đôi Hunter, người đạt 45 điểm trong bài kiểm tra toán. Điểm kiểm tra của Grant là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
           <t>Nếu Hunter đạt điểm 45 trong bài kiểm tra toán thì John nhận được số điểm gấp đôi nên John đạt 45 x 2 = 90 điểm. Grant ghi được nhiều hơn John 10 điểm nên Grant ghi được 90 + 10 = 100 điểm. Vì vậy, điểm kiểm tra của Grant là 100. #### 100 Đáp án là: 100</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Jimmy muốn chơi trong bể bơi bơm hơi ở sân sau nhà mình. Bể bơi trống rỗng và gara bị khóa nên anh ta không thể dùng vòi để đổ nước vào bể. Anh ta tìm một cái xô 2 gallon và tính rằng phải mất 20 giây để đổ đầy nước từ vòi và mang nó đến bể nơi anh ta đổ nước vào. Nếu hồ chứa 84 gallon nước thì Jimmy sẽ mất bao nhiêu phút để đổ đầy hồ?</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Jimmy có thể đổ đầy bể bằng một thùng 2 gallon, vì vậy anh ta sẽ cần đổ đầy thùng 84/2 = 42 lần để đổ đầy bể. Jimmy mất 20 giây để đổ đầy thùng, do đó anh ấy sẽ mất 20 * 42 = 840 giây để đổ đầy bể. Vì một phút có 60 giây nên Jimmy sẽ mất 840/60 = 14 phút để làm đầy bể. ####14 Đáp án là: 14</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Nếu Brenda và chín người bạn của cô ấy dự định đặt một chiếc pizza, và mỗi người dự định ăn 2 lát, và mỗi chiếc pizza có 4 lát, thì họ nên đặt bao nhiêu chiếc pizza?</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Brenda và 9 người bạn của cô ấy có tổng cộng 9 + 1 = 10 người. Mỗi người dự định ăn 2 lát nên sẽ cần tổng cộng 10 x 2 = 20 lát. Mỗi chiếc pizza có 4 lát nên họ sẽ cần đặt 20/4 = 5 chiếc pizza. ####5 Đáp án là: 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Một học sinh trong chuyến đi thực tế đã đếm được 12 con sóc. Một em khác đếm được số sóc nhiều hơn học sinh thứ nhất một phần ba. Cả hai học sinh đã đếm được tổng cộng bao nhiêu con sóc?</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Học sinh đầu tiên đếm được 12 con sóc. Học sinh thứ hai đếm được nhiều con sóc hơn học sinh thứ nhất một phần ba, nghĩa là nhiều hơn 1/3 * 12 = 4 con sóc. Vậy học sinh thứ hai đếm được 12 + 4 = 16 con sóc. Cộng lại, cả hai học sinh đếm được 12 + 16 = 28 con sóc. ####28 Đáp án là: 28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
22-04_14-53 Optimize module-4 exercise for speed and accuracy
</commit_message>
<xml_diff>
--- a/data/sample_dataset.xlsx
+++ b/data/sample_dataset.xlsx
@@ -1,34 +1,109 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ngocduy/TTTH/llm-application-programming-course/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF287F5F-8DA1-6F45-BC2D-E0AB4FFE3F5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="40960" windowHeight="25000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+  <si>
+    <t>query_vi</t>
+  </si>
+  <si>
+    <t>response_vi</t>
+  </si>
+  <si>
+    <t>Forest và những người bạn của anh ấy đã chuẩn bị một chiếc bánh sinh nhật cho người bạn Juelz của họ có 240 chiếc bánh. Sau khi hát bài hát sinh nhật, họ đã ăn 60% số miếng bánh và sau đó, Juelz chia những miếng còn lại cho ba chị em của mình. Hỏi mỗi chị em nhận được bao nhiêu miếng bánh?</t>
+  </si>
+  <si>
+    <t>Ban đầu có 240 miếng bánh. Họ ăn 60% số bánh nên họ ăn 240 * 0,60 = 144 miếng. Số miếng bánh còn lại là 240 - 144 = 96 miếng. Juelz chia phần còn lại cho ba chị em mình nên mỗi chị em nhận được 96/3 = 32 miếng bánh. ####32 Đáp án là: 32</t>
+  </si>
+  <si>
+    <t>Nếu một vườn thú có 21 con chim cánh cụt và số gấu Bắc Cực nhiều gấp đôi thì tổng số động vật trong vườn thú là bao nhiêu?</t>
+  </si>
+  <si>
+    <t>Nếu vườn thú có 21 con chim cánh cụt thì nó có 2*21 = 42 con gấu Bắc Cực. Tổng số động vật trong vườn thú là 21 con chim cánh cụt + 42 con gấu bắc cực = 63 con. ####63 Đáp án là: 63</t>
+  </si>
+  <si>
+    <t>Trong lớp của thầy Abraham, $10$ trong số học sinh $15$ đã nhận được $A$ trong bài kiểm tra mới nhất. Nếu cùng tỷ lệ học sinh nhận được $A$ trong bài kiểm tra mới nhất của bà Berkeley và nếu bà Berkeley có tổng số học sinh là $24$ thì có bao nhiêu học sinh trong lớp của bà Berkeley nhận được $A$?</t>
+  </si>
+  <si>
+    <t>Nếu $10$ trên tổng số $15$ học sinh nhận được $A$ trong lớp của thầy Abraham thì tỷ lệ học sinh nhận được $A$ là $\frac{10}{15}=\frac{2}{3}$ . Nếu cùng một tỷ lệ học sinh nhận được $A$ trong lớp của cô Berkeley, thì $\frac{2}{3}$ trong số học sinh $24$ của cô nhận được $A$, tức là $\frac{2}{3} \cdot24=\boxed{16}$ sinh viên. Đáp án là: 16</t>
+  </si>
+  <si>
+    <t>Nina muốn tặng quà cho các con của cô ấy. Cô ấy mua ba món đồ chơi với giá 10 đô la mỗi cái, hai gói thẻ bóng rổ với giá 5 đô la mỗi chiếc và năm chiếc áo sơ mi với giá 6 đô la mỗi chiếc. Tổng cộng cô ấy chi bao nhiêu?</t>
+  </si>
+  <si>
+    <t>Nina mua 3 món đồ chơi với giá 10 USD mỗi món, vì vậy cô ấy chi 3*10 = 30 USD cho đồ chơi. Cô ấy mua 2 gói thẻ bóng rổ với giá 5 đô la mỗi gói, vì vậy cô ấy chi 2 * 5 = 10 đô la cho thẻ bóng rổ. Cô ấy mua 5 chiếc áo sơ mi với giá 6 đô la mỗi chiếc, vì vậy cô ấy chi 5 * 6 = 30 đô la cho chiếc áo sơ mi. Tổng cộng, cô ấy chi 30+10+30 = 70$. #### 70 Đáp án là: 70</t>
+  </si>
+  <si>
+    <t>Phải mất bốn họa sĩ làm việc với cùng mức lương $1,25$ ngày làm việc để hoàn thành một công việc. Nếu chỉ có ba người thợ sơn thì họ sẽ hoàn thành công việc với tốc độ như nhau trong bao nhiêu ngày công? Thể hiện câu trả lời của bạn dưới dạng số hỗn hợp.</t>
+  </si>
+  <si>
+    <t>Nếu bốn họa sĩ làm việc với cùng một mức lương là $1,25$ ngày công để hoàn thành công việc thì tổng số công việc cần thiết cho công việc là $4\cdot 1,25=5$ ngày công. Vì giả định mức lương như nhau cho tất cả các họa sĩ, nên chúng ta có thể nói rằng ba họa sĩ làm việc với cùng một mức lương sẽ mất $5/3=\boxed{1\frac{2}{3}}$ ngày làm việc để hoàn thành công việc. Câu trả lời là: 1\frac{2}{3}</t>
+  </si>
+  <si>
+    <t>Đặt $\mathbf{v__0$ là một vectơ. Vectơ $\mathbf{v} _0$ được chiếu lên $\begin{pmatrix} 3 \\ 1 \end{pmatrix},$ tạo thành vectơ $\mathbf{v__1.$ Vectơ $\mathbf{v Sau đó, _1$ được chiếu lên $\begin{pmatrix} X \\ 1 \end{pmatrix},$ tạo thành vectơ $\mathbf{v} _2.$ Tìm ma trận nhận $\mathbf{v__0$ tới $\mathbf{v&gt;&lt;/2. 5. Giá trị của biến X chưa biết là bao nhiêu?</t>
+  </si>
+  <si>
+    <t>Để giải quyết vấn đề này, chúng ta cần xác định ma trận đưa $\mathbf{v&gt;&lt;/0$ đến $\mathbf{v&gt;&lt;/2.$ Đặt $\mathbf{v__0 = \begin{pmatrix} a \\ b \ end{pmatrix}.$ Phép chiếu của $\mathbf{v&gt;&lt;/0$ lên $\begin{pmatrix} 3 \\ 1 \end{pmatrix}$ được đưa ra bởi \[\operatorname{proj__{\begin{pmatrix } 3 \\ 1 \end{pmatrix}} \mathbf{v__0 = \frac{\begin{pmatrix} a \\ b \end{pmatrix} \cdot \begin{pmatrix} 3 \\ 1 \end{pmatrix }}{\begin{pmatrix} 3 \\ 1 \end{pmatrix} \cdot \begin{pmatrix} 3 \\ 1 \end{pmatrix}} \begin{pmatrix} 3 \\ 1 \end{pmatrix} = \ frac{3a + b}{10} \begin{pmatrix} 3 \\ 1 \end{pmatrix}.\]Cho $\mathbf{v} _1 = \frac{3a + b}{10} \begin{pmatrix} 3 \\ 1 \end{pmatrix}.$ Phép chiếu của $\mathbf{v&gt;&lt;/1$ lên $\begin{pmatrix} X \\ 1 \end{pmatrix}$ được cho bởi \[\operatorname{proj&gt;&lt;/ {\begin{pmatrix} X \\ 1 \end{pmatrix}} \mathbf{v} _1 = \frac{\frac{3a + b}{10} \begin{pmatrix} 3 \\ 1 \end{pmatrix} \cdot \begin{pmatrix} X \\ 1 \end{pmatrix}}{\begin{pmatrix} X \\ 1 \end{pmatrix} \cdot \begin{pmatrix} X \\ 1 \end{pmatrix}} \ started{pmatrix} X \\ 1 \end{pmatrix} = \frac{(3a + b)(3X + 1)}{10(X^2 + 1)} \begin{pmatrix} X \\ 1 \end{ pmatrix}.\]Cho $\mathbf{v y2 = \frac{(3a + b)(3X + 1)}{10(X^2 + 1)} \begin{pmatrix} X \\ 1 \end{ pmatrix}.$ Do đó, ma trận lấy $\mathbf{v} _0$ đến $\mathbf{v} _2$ là \[\boxed{\begin{pmatrix} \frac{(3X + 1)(3a + b )}{10(X^2 + 1)} \\ \frac{(3a + b)}{10(X^2 + 1)} \end{pmatrix}}.\] Đáp án là: 1</t>
+  </si>
+  <si>
+    <t>Các trinh sát ngoài trời đã đi bộ đường dài để xem thác nước. Để đi bộ đường dài, các thành viên câu lạc bộ đã đi 3 ô tô, 6 taxi và 2 xe tải. Mỗi ô tô có 4 người, mỗi xe taxi có 6 người và mỗi xe tải có 5 người. Có bao nhiêu người đã đi leo núi?</t>
+  </si>
+  <si>
+    <t>Trên xe có 3 ô tô * 4 người = 12 người. Trên xe có 6 chiếc taxi * 6 người = 36 người. Có 2 xe * 5 người = 10 người trên xe. Vậy tổng cộng có 12 + 36 + 10 = 58 người đã đi bộ đường dài. ####58 Đáp án là: 58</t>
+  </si>
+  <si>
+    <t>Trong vòng ba ngày, Markeesha đã bán được 30 hộp bánh quy giòn vào thứ Sáu để gây quỹ cho đội trinh sát của cô. Ngày thứ bảy, số hộp cô bán được gấp đôi ngày thứ sáu. Vào Chủ Nhật, cô bán được ít hơn 15 hộp so với thứ Bảy. Markeesha đã bán tổng cộng bao nhiêu hộp trong ba ngày?</t>
+  </si>
+  <si>
+    <t>Vào thứ Sáu, Markeesha đã bán được 30 hộp bánh quy giòn. Ngày thứ bảy cô bán được số hộp gấp đôi ngày thứ sáu nên cô bán được 2 * 30 = 60 hộp. Chủ nhật cô bán ít hơn ngày thứ bảy 15 hộp nên cô bán được 60 - 15 = 45 hộp. Tổng cộng, Markeesha đã bán được 30 + 60 + 45 = 135 hộp trong ba ngày. ####135 Đáp án là: 135</t>
+  </si>
+  <si>
+    <t>Charley đã mua 30 cây bút chì. Cô đã đánh mất 6 cây bút chì khi chuyển đến trường, và tất nhiên, cô cũng làm mất 1/3 số bút chì còn lại vì cô không giỏi theo dõi bút chì. Hiện tại cô ấy có bao nhiêu cây bút chì?</t>
+  </si>
+  <si>
+    <t>Charley đã mua 30 cây bút chì. Cô ấy làm mất 6 chiếc bút chì nên cô ấy còn lại 30 - 6 = 24 chiếc bút chì. Cô mất 1/3 số bút chì còn lại nên cô mất 1/3 * 24 = 8 chiếc bút chì. Vậy hiện tại cô có 24 - 8 = 16 chiếc bút chì. ####16 Đáp án là: 16</t>
+  </si>
+  <si>
+    <t>Tom thuê một chiếc trực thăng 2 giờ mỗi ngày trong 3 ngày. Giá thuê là 75 USD một giờ. Anh ấy đã trả bao nhiêu?</t>
+  </si>
+  <si>
+    <t>Tom thuê chiếc trực thăng 2 giờ mỗi ngày trong 3 ngày, vậy anh ấy thuê nó với tổng số tiền là 2 * 3 = 6 giờ. Chi phí thuê trực thăng là 75 USD một giờ, vậy tổng chi phí là 6 * 75 USD = 450 USD. Tom đã trả 450 đô la để thuê chiếc trực thăng. ####450 Đáp án là: 450</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,80 +122,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,144 +424,96 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>query_vi</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>response_vi</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Tiệm bánh pizza bán pizza nhỏ với giá 2 đô la và pizza lớn với giá 8 đô la. Họ đã bán được 40 đô la tiền pizza. Nếu họ bán 8 chiếc pizza nhỏ thì họ đã bán được bao nhiêu chiếc pizza lớn?</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Nếu tiệm bánh pizza bán 8 chiếc pizza nhỏ với giá 2 đô la mỗi chiếc thì họ kiếm được 8 * 2 đô la = 16 đô la từ những chiếc pizza nhỏ. Họ đã bán được tổng cộng 40 đô la tiền pizza, vì vậy số tiền còn lại phải đến từ những chiếc pizza lớn. Số tiền làm được từ những chiếc pizza lớn là $40 - $16 = $24. Vì mỗi chiếc bánh pizza lớn có giá 8 đô la nên họ phải bán được 24 đô la / 8 đô la = 3 chiếc bánh pizza lớn. Vì vậy, họ đã bán được 3 chiếc pizza lớn. ####3 Đáp án là: 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Sau khi nướng 200 chiếc bánh nhân thịt trong một ngày và bán với giá 20 USD mỗi chiếc, Du Chin dùng 3/5 số tiền bán được để mua nguyên liệu làm bánh nhân thịt cho ngày hôm sau. Đỗ Chín còn lại bao nhiêu tiền sau khi dành tiền mua nguyên liệu?</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Du Chin bán 200 cái bánh nhân thịt với giá 20$ mỗi cái, vậy tổng doanh thu là 200 x 20$ = $&lt;&lt;200*20=4000&gt;&gt;4000. Anh ấy sử dụng 3/5 doanh số bán hàng để mua nguyên liệu, vì vậy anh ấy chi 3/5 x $4000 = $&lt;&lt;3/5*4000=2400&gt;&gt;2400 cho nguyên liệu. Vì vậy, Du Chin còn lại $4000 - $2400 = $&lt;&lt;4000-2400=1600&gt;&gt;1600 sau khi dành tiền mua nguyên liệu. ####1600 Đáp án là: 1600</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Trung bình của $x+6$, $6x+2$ và $2x+7$ là $4x-7$. $x$ là gì?</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Trung bình cộng của ba số được tìm thấy bằng cách cộng chúng lại và chia cho 3. Vì vậy, chúng ta có phương trình: \[\frac{(x+6) + (6x+2) + (2x+7)}{3} = 4x-7.\] Rút gọn vế trái, ta có: \[\frac{9x+15}{3} = 4x-7.\] Nhân cả hai vế với 3 để loại bỏ phân số, ta có: \[ 9x+15 = 12x-21.\] Trừ 9x ở cả hai vế, ta có: \[15 = 3x-21.\] Cộng 21 vào cả hai vế, ta có: \[36 = 3x.\] Chia cả hai vế cho 3, ta có: \[x = 12.\] Vậy giá trị của x là $\boxed{12}$.Câu trả lời là: 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Trong tháng đầu năm, các gia đình đến thăm công viên quốc gia đã nhìn thấy động vật 26 lần. Trong tháng thứ hai, số lần nhìn thấy động vật nhiều gấp ba lần so với tháng Giêng. Trong tháng thứ ba, số lần nhìn thấy động vật giảm xuống còn một nửa so với tháng thứ hai. Tổng số lần các gia đình nhìn thấy một con vật trong ba tháng đầu năm là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Trong tháng đầu tiên, các gia đình đã nhìn thấy động vật 26 lần. Trong tháng thứ hai, số lần nhìn thấy động vật nhiều gấp ba lần so với tháng đầu tiên, do đó 26 x 3 = 78 lần nhìn thấy động vật. Trong tháng thứ ba, số lần nhìn thấy động vật giảm xuống còn một nửa so với tháng thứ hai, do đó 78/2 = 39 lần nhìn thấy động vật. Tổng số lần gia đình nhìn thấy một con vật trong 3 tháng đầu năm là 26 + 78 + 39 = 143. #### 143 Đáp án là: 143</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Keenan cần viết một bài luận dài 1200 từ. Bài luận của cô ấy sẽ đến hạn vào lúc nửa đêm. Cô ấy viết 400 từ mỗi giờ trong hai giờ đầu tiên. Sau đó, cô viết 200 từ mỗi giờ. Cô ấy cần bắt đầu hoàn thành đúng thời hạn bao nhiêu giờ trước thời hạn?</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Keenan viết 400 từ mỗi giờ trong 2 giờ đầu, vậy cô ấy viết 400 x 2 = 800 từ trong 2 giờ đầu. Cô ấy cần viết tổng cộng 1200 từ, vậy cô ấy còn 1200 - 800 = 400 từ để viết. Sau 2 giờ đầu, cô ấy viết được 200 từ mỗi giờ, vậy cô ấy cần 400/200 = 2 giờ nữa để viết xong. Vì vậy, cô ấy cần bắt đầu viết trước thời hạn 2 + 2 = 4 tiếng để hoàn thành đúng hạn. ####4 Đáp án là: 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Cho rằng (3,17) và (9,-4) là hai đỉnh đối diện của một hình chữ nhật, tổng tọa độ y của hai đỉnh còn lại là bao nhiêu?</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Các đỉnh đối diện của hình chữ nhật cách đều tâm hình chữ nhật. Tâm của hình chữ nhật là trung điểm của đoạn thẳng nối hai đỉnh đối diện. Trung điểm của đoạn thẳng nối (3,17) và (9,-4) là $\left(\frac{3+9}{2},\frac{17+(-4)}{2}\right ) = (6, \frac{13}{2})$. Hai đỉnh còn lại của hình chữ nhật cũng cách đều tâm hình chữ nhật. Do đó, tổng tọa độ y của hai đỉnh còn lại là $2 \times \frac{13}{2} = \boxed{13}$. Câu trả lời là: 13</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Harry đang đi xe buýt về nhà. Anh ấy đã ngồi trên xe buýt được 15 phút và anh ấy biết chặng đường còn lại sẽ mất thêm 25 phút nữa. Quãng đường đi bộ từ bến xe buýt đến nhà anh ấy sẽ mất một nửa thời gian so với thời gian đi xe buýt. Tổng cộng Harry sẽ dành bao nhiêu phút để đi du lịch?</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Harry đã ở trên xe buýt được 15 phút rồi. Phần còn lại của hành trình xe buýt sẽ mất thêm 25 phút nữa. Cho đến nay, Harry đã đi xe buýt tổng cộng 15 + 25 = 40 phút. Quãng đường đi bộ từ bến xe buýt đến nhà anh ấy sẽ mất một nửa thời gian so với thời gian đi xe buýt. Một nửa của 40 phút là 40/2 = 20 phút. Tổng cộng Harry sẽ mất 40 phút đi xe buýt + 20 phút đi bộ = 60 phút di chuyển. ####60 Đáp án là: 60</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Jimmy muốn chơi trong bể bơi bơm hơi ở sân sau nhà mình. Bể bơi trống rỗng và gara bị khóa nên anh ta không thể dùng vòi để đổ nước vào bể. Anh ta tìm một cái xô 2 gallon và tính rằng phải mất 20 giây để đổ đầy nước từ vòi và mang nó đến bể nơi anh ta đổ nước vào. Nếu hồ chứa 84 gallon nước thì Jimmy sẽ mất bao nhiêu phút để đổ đầy hồ?</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Jimmy có thể đổ đầy bể bằng một thùng 2 gallon, vì vậy anh ta sẽ cần đổ đầy thùng 84/2 = 42 lần để đổ đầy bể. Jimmy mất 20 giây để đổ đầy thùng, do đó anh ấy sẽ mất 20 * 42 = 840 giây để đổ đầy bể. Vì một phút có 60 giây nên Jimmy sẽ mất 840/60 = 14 phút để làm đầy bể. ####14 Đáp án là: 14</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Jenna đang viền chiếc váy dạ hội của mình. Viền váy dài 3 feet. Mỗi mũi khâu mà Jenna thực hiện dài 1/4 inch. Nếu Jenna khâu 24 mũi mỗi phút thì Jenna mất bao nhiêu phút để viền váy?</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Đầu tiên, chúng ta cần chuyển đổi chiều dài của viền váy từ feet sang inch. Vì có 12 inch trong một foot nên chiều dài của viền áo tính bằng inch là 3 feet * 12 inch/foot = 36 inch. Tiếp theo, chúng ta cần tìm hiểu xem Jenna cần thực hiện bao nhiêu mũi khâu để viền chiếc váy. Vì mỗi mũi khâu dài 1/4 inch nên số mũi khâu cần thiết là 36 inch / (1/4 inch/mũi) = 36 inch * (4 mũi/1 inch) = 144 mũi. Cuối cùng, chúng ta cần xác định Jenna phải mất bao nhiêu phút để thực hiện 144 mũi khâu. Nếu Jenna thực hiện 24 mũi khâu mỗi phút thì cô ấy sẽ phải mất 144 mũi khâu / 24 mũi khâu/phút = 6 phút để viền váy. ####6 Đáp án là: 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Nếu Brenda và chín người bạn của cô ấy dự định đặt một chiếc pizza, và mỗi người dự định ăn 2 lát, và mỗi chiếc pizza có 4 lát, thì họ nên đặt bao nhiêu chiếc pizza?</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Brenda và 9 người bạn của cô ấy có tổng cộng 9 + 1 = 10 người. Mỗi người dự định ăn 2 lát nên sẽ cần tổng cộng 10 x 2 = 20 lát. Mỗi chiếc pizza có 4 lát nên họ sẽ cần đặt 20/4 = 5 chiếc pizza. ####5 Đáp án là: 5</t>
-        </is>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>